<commit_message>
fix: enforce position recovery checkpoints
</commit_message>
<xml_diff>
--- a/assets/中台网关原始出账订单.xlsx
+++ b/assets/中台网关原始出账订单.xlsx
@@ -543,7 +543,8 @@
     <col min="12" max="12" width="14" style="1" customWidth="1"/>
     <col min="13" max="17" width="14" customWidth="1"/>
     <col min="18" max="20" width="16" customWidth="1"/>
-    <col min="21" max="22" width="14" customWidth="1"/>
+    <col min="21" max="21" width="14" style="1" customWidth="1"/>
+    <col min="22" max="22" width="14" customWidth="1"/>
     <col min="23" max="23" width="14" style="1" customWidth="1"/>
     <col min="24" max="24" width="14" customWidth="1"/>
     <col min="25" max="25" width="18" style="1" customWidth="1"/>
@@ -614,7 +615,7 @@
       <c r="T1" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="U1" s="2" t="s">
+      <c r="U1" s="3" t="s">
         <v>20</v>
       </c>
       <c r="V1" s="2" t="s">

</xml_diff>